<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-06 Amir dit stop
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-06.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le coussin chat</t>
+          <t>Amir dit stop</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon</t>
+          <t>salon, table, lampe, fenêtre, cadre, coussin, sol, orange, mur, bol</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, Aniss, maman</t>
+          <t>Amir, Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina joue avec le coussin chat. Aniss le met trop près. Nina dit stop, s'éloigne, rejoint maman. Le coussin reste loin.</t>
+          <t>Ça sent l'orange près de la table. Sur le mur, un éclat de cadre luit. Amir veut jouer, maintenant. Nina met le coussin trop près. Sourire parti. Papa s'accroupit. Stop, un pas. Merci vécu. Deuxième ruse : le coussin glisse. Un éclat de cadre tient sur le mur.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les volets font des rayures. Le soleil est sur le canapé. Ça sent le pain grillé. L'horloge fait tic tac. Un gros coussin est là. Il a une tête de chat. Il est doux et gros. Tu as vu le coussin chat, Nina ? Oui, maman. Il est doux. Il sent la lessive. En ce moment, Nina joue. Aniss joue avec elle. Ils sont au salon. Aniss met le coussin trop près. Le coussin appuie sur Nina. Nina est gênée. Le coussin est trop près. Son ventre se serre. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Nina fait un pas. Elle peut s'éloigner. Elle s'éloigne vers maman. Maman est l'adulte sur le canapé. Maman, c'est trop. Tu as dit stop. Bravo, Nina. Tu t'es éloignée. Tu es venue vers moi. Le coussin reste loin, d'accord ? D'accord. Nina reste près d'elle. Elle souffle. Le coussin reste loin. Stop, puis on s'éloigne. Puis on va vers un adulte. Aniss pose le coussin chat au sol. Nina se sent plus calme. Les rayures des volets bougent. Elles avancent sur le canapé. Tu as vu le soleil bouger ? Oui. Il avance. Ça sent encore le pain grillé. Nina pose sa main sur le canapé. Le tissu est chaud. On reste ici un moment ? Oui, maman.</t>
+          <t>Ça sent l'orange, près de la table. Ça sent bon, papa. Tu le sens, le fruit ouvert ? Oui, papa. Le jus brille un peu. J'ai ouvert l'orange. Elle brille, maman. Maman pose le bol rond. Le bol est froid, un peu lisse. Il est froid. Tu le touches, Amir ? Oui, du doigt. Sur le mur, un éclat de cadre luit. Il brille, maman. Tu le vois, sur le verre ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bois. Le bois de la table gratte un peu. Il gratte, papa. Tu t'assois, Amir ? Un peu. Une peau d'orange dort sur le bois. Une peau, maman. Elle est sèche ? Oui. La lampe chauffe le mur, tout près. Elle chauffe, papa. Tu la sens, la lampe ? Oui, elle chauffe. Une goutte tombe dans le bol. Ploc. C'est une goutte. Les pieds d'Amir touchent le sol. Mes pieds, papa. Tu es bien assis, Amir ? Oui, papa. Le sol est lisse, un peu froid. Il est lisse. Nina arrive près de la table. Ses pieds glissent sur le bois. Le coussin. Tu viens, Nina ? Oui. Maman pose le gros coussin. Il est mou, un peu lourd. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. En ce moment, Amir tend le coussin. Tu le donnes à Nina ? Oui, maman. Nina prend le coussin. Elle le met trop près. Près. Le coussin appuie sur Amir. Oh. Nina pousse plus fort. Joue. Amir baisse les yeux. Le sourire d'Amir disparaît. Dans sa poitrine, ça se serre. L'envie et l'inquiétude se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu es serré, Amir ? Un peu, papa. Tes mains sont froides, Amir ? Un peu, maman. L'éclat de cadre tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les volets font des rayures. Le soleil est sur le canapé. Ça sent le pain grillé. L'horloge fait tic tac. Un gros coussin est là. Il a une tête de chat. Il est doux et gros. Tu as vu le coussin chat, Nina ? Oui, maman. Il est doux. Il sent la lessive. En ce moment, Nina joue. Aniss joue avec elle. Ils sont au salon. Aniss met le coussin trop près. Le coussin appuie sur Nina. Nina est gênée. Le coussin est trop près. Son ventre se serre. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Nina fait un pas. Elle peut s'éloigner. Elle s'éloigne vers maman. Maman est l'adulte sur le canapé. Maman, c'est trop. Tu as dit stop. Bravo, Nina. Tu t'es éloignée. Tu es venue vers moi. Le coussin reste loin, d'accord ? D'accord. Nina reste près d'elle. Elle souffle. Le coussin reste loin. Stop, puis on s'éloigne. Puis on va vers un adulte. Aniss pose le coussin chat au sol. Nina se sent plus calme. Les rayures des volets bougent. Elles avancent sur le canapé. Tu as vu le soleil bouger ? Oui. Il avance. Ça sent encore le pain grillé. Nina pose sa main sur le canapé. Le tissu est chaud. On reste ici un moment ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ça sent l'orange, près de la table. Ça sent bon, papa. Tu le sens, le fruit ouvert ? Oui, papa. Le jus brille un peu. J'ai ouvert l'orange. Elle brille, maman. Maman pose le bol rond. Le bol est froid, un peu lisse. Il est froid. Tu le touches, Amir ? Oui, du doigt. Sur le mur, un &lt;emphasis level="moderate"&gt;éclat de cadre&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le verre ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bois. Le bois de la table gratte un peu. Il gratte, papa. Tu t'assois, Amir ? Un peu. Une peau d'orange dort sur le bois. Une peau, maman. Elle est sèche ? Oui. La lampe chauffe le mur, tout près. Elle chauffe, papa. Tu la sens, la lampe ? Oui, elle chauffe. Une goutte tombe dans le bol. Ploc. C'est une goutte. Les pieds d'Amir touchent le sol. Mes pieds, papa. Tu es bien assis, Amir ? Oui, papa. Le sol est lisse, un peu froid. Il est lisse. Nina arrive près de la table. Ses pieds glissent sur le bois. Le coussin. Tu viens, Nina ? Oui. Maman pose le gros coussin. Il est mou, un peu lourd. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. En ce moment, Amir tend le coussin. Tu le donnes à Nina ? Oui, maman. Nina prend le coussin. Elle le met trop près. Près. Le coussin appuie sur Amir. Oh. Nina pousse plus fort. Joue. Amir baisse les yeux. Le sourire d'Amir disparaît. Dans sa poitrine, ça se serre. L'envie et l'inquiétude se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu es serré, Amir ? Un peu, papa. Tes mains sont froides, Amir ? Un peu, maman. L'éclat de cadre tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;François joue dans le salon. Maman est sur le canapé. Nina met un coussin trop près. C'est trop. François dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il fait un pas. Il peut s'éloigner. Il s'éloigne vers maman. Maman est l'adulte. François dit : maman, c'est trop. Maman écoute. François reste près d'elle. Maman dit : stop, puis on s'éloigne. Puis on va vers un adulte. François souffle. Le coussin reste loin. François se sent plus calme.&lt;/slow&gt; [pause]</t>
+          <t>Ça sent l'orange, près de la table. Ça sent bon, papa. Tu le sens, le fruit ouvert ? Oui, papa. Le jus brille un peu. J'ai ouvert l'orange. Elle brille, maman. Maman pose le bol rond. Le bol est froid, un peu lisse. Il est froid. Tu le touches, Amir ? Oui, du doigt. Sur le mur, un &lt;emphasis&gt;éclat de cadre&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le verre ? Oui, un petit point. Le soleil le touche. Un rayon glisse sur le bois. Le bois de la table gratte un peu. Il gratte, papa. Tu t'assois, Amir ? Un peu. Une peau d'orange dort sur le bois. Une peau, maman. Elle est sèche ? Oui. La lampe chauffe le mur, tout près. Elle chauffe, papa. Tu la sens, la lampe ? Oui, elle chauffe. Une goutte tombe dans le bol. Ploc. C'est une goutte. Les pieds d'Amir touchent le sol. Mes pieds, papa. Tu es bien assis, Amir ? Oui, papa. Le sol est lisse, un peu froid. Il est lisse. Nina arrive près de la table. Ses pieds glissent sur le bois. Le coussin. Tu viens, Nina ? Oui. Maman pose le gros coussin. Il est mou, un peu lourd. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. En ce moment, Amir tend le coussin. Tu le donnes à Nina ? Oui, maman. Nina prend le coussin. Elle le met trop près. Près. Le coussin appuie sur Amir. Oh. Nina pousse plus fort. Joue. Amir baisse les yeux. Le sourire d'Amir disparaît. Dans sa poitrine, ça se serre. L'envie et l'inquiétude se heurtent. Ses épaules montent un peu. Papa s'accroupit à la même hauteur. Tu es serré, Amir ? Un peu, papa. Tes mains sont froides, Amir ? Un peu, maman. L'éclat de cadre tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de cadre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,60 +1324,85 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis gêne; intensite=2; destinataire=enfant; sous_texte=il_veut_jouer_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les volets font des rayures.
-narrateur|Le soleil est sur le canapé.
-narrateur|Ça sent le pain grillé.
-narrateur|L'horloge fait tic tac.
-narrateur|Un gros coussin est là.
-narrateur|Il a une tête de chat.
-narrateur|Il est doux et gros.
-maman|Tu as vu le coussin chat, Nina ?
-enfant-f|Oui, maman. Il est doux.
-maman|Il sent la lessive.
-narrateur|En ce moment, Nina joue.
-narrateur|Aniss joue avec elle.
-narrateur|Ils sont au salon.
-narrateur|Aniss met le coussin trop près.
-narrateur|Le coussin appuie sur Nina.
-narrateur|Nina est gênée.
-narrateur|Le coussin est trop près.
-narrateur|Son ventre se serre.
-narrateur|Ses épaules montent.
-enfant-f|Je n'aime pas.
-enfant-f|C'est trop.
-enfant-f|Stop.
-narrateur|Nina fait un pas.
-narrateur|Elle peut s'éloigner.
-narrateur|Elle s'éloigne vers maman.
-narrateur|Maman est l'adulte sur le canapé.
-enfant-f|Maman, c'est trop.
-maman|Tu as dit stop.
-maman|Bravo, Nina.
-maman|Tu t'es éloignée.
-maman|Tu es venue vers moi.
-maman|Le coussin reste loin, d'accord ?
-enfant-f|D'accord.
-narrateur|Nina reste près d'elle.
-narrateur|Elle souffle.
-narrateur|Le coussin reste loin.
-maman|Stop, puis on s'éloigne.
-maman|Puis on va vers un adulte.
-narrateur|Aniss pose le coussin chat au sol.
-narrateur|Nina se sent plus calme.
-narrateur|Les rayures des volets bougent.
-narrateur|Elles avancent sur le canapé.
-maman|Tu as vu le soleil bouger ?
-enfant-f|Oui. Il avance.
-narrateur|Ça sent encore le pain grillé.
-narrateur|Nina pose sa main sur le canapé.
-narrateur|Le tissu est chaud.
-maman|On reste ici un moment ?
-enfant-f|Oui, maman.</t>
+          <t>narrateur|Ça sent l'orange, près de la table.
+enfant-m|Ça sent bon, papa.
+papa|Tu le sens, le fruit ouvert ?
+enfant-m|Oui, papa.
+narrateur|Le jus brille un peu.
+maman|J'ai ouvert l'orange.
+enfant-m|Elle brille, maman.
+narrateur|Maman pose le bol rond.
+narrateur|Le bol est froid, un peu lisse.
+enfant-m|Il est froid.
+papa|Tu le touches, Amir ?
+enfant-m|Oui, du doigt.
+narrateur|Sur le mur, un éclat de cadre luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le verre ?
+enfant-m|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse sur le bois.
+narrateur|Le bois de la table gratte un peu.
+enfant-m|Il gratte, papa.
+maman|Tu t'assois, Amir ?
+enfant-m|Un peu.
+narrateur|Une peau d'orange dort sur le bois.
+enfant-m|Une peau, maman.
+maman|Elle est sèche ?
+enfant-m|Oui.
+narrateur|La lampe chauffe le mur, tout près.
+enfant-m|Elle chauffe, papa.
+papa|Tu la sens, la lampe ?
+enfant-m|Oui, elle chauffe.
+narrateur|Une goutte tombe dans le bol.
+enfant-m|Ploc.
+maman|C'est une goutte.
+narrateur|Les pieds d'Amir touchent le sol.
+enfant-m|Mes pieds, papa.
+papa|Tu es bien assis, Amir ?
+enfant-m|Oui, papa.
+narrateur|Le sol est lisse, un peu froid.
+enfant-m|Il est lisse.
+narrateur|Nina arrive près de la table.
+narrateur|Ses pieds glissent sur le bois.
+copine|Le coussin.
+enfant-m|Tu viens, Nina ?
+copine|Oui.
+narrateur|Maman pose le gros coussin.
+narrateur|Il est mou, un peu lourd.
+enfant-m|Je veux jouer, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|En ce moment, Amir tend le coussin.
+maman|Tu le donnes à Nina ?
+enfant-m|Oui, maman.
+narrateur|Nina prend le coussin.
+narrateur|Elle le met trop près.
+copine|Près.
+narrateur|Le coussin appuie sur Amir.
+enfant-m|Oh.
+narrateur|Nina pousse plus fort.
+copine|Joue.
+narrateur|Amir baisse les yeux.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, ça se serre.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Ses épaules montent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu es serré, Amir ?
+enfant-m|Un peu, papa.
+maman|Tes mains sont froides, Amir ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de cadre tremble, puis tient.</t>
         </is>
       </c>
     </row>
@@ -1404,17 +1429,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Nina. Que fait-elle ?</t>
+          <t>C'est trop pour Amir. Que fait-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Nina. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est &lt;emphasis level="moderate"&gt;trop&lt;/emphasis&gt; pour Amir. Que fait-il ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est trop pour François. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est &lt;emphasis&gt;trop&lt;/emphasis&gt; pour Amir. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1477,7 +1502,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1488,7 +1513,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1503,34 +1528,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>trop</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1545,7 +1574,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1555,12 +1584,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=c_est_trop_pour_amir_que_fait_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Nina. Que fait-elle ?</t>
+          <t>narrateur|C'est trop pour Amir.
+narrateur|Que fait-il ?</t>
         </is>
       </c>
     </row>
@@ -1587,17 +1617,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina a dit stop. Elle a pu s'éloigner. Elle est allée vers maman, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. Le coussin chat est loin. L'horloge fait tic tac.</t>
+          <t>Amir veut jouer, tout de suite. Je joue, maintenant ! Il avance trop vite vers Nina. Le coussin reste collé à sa poitrine. Viens. Nina pousse le coussin. Oh. Le sourire ne revient pas. C'est trop. Stop. Amir recule d'un pas. Personne ne parle. Il observe le coussin, un instant. Il écoute le bruit de la lampe. Tu veux de l'air, Amir ? Papa reste à la même hauteur. Plus loin. Nina ne dit rien, d'abord. Elle tire le coussin vers elle. Loin. Loin, oui. Merci, Amir. Papa a vu les deux, près du bol. Le coussin colle un peu, sous les doigts. Il est mou. Nina pose le coussin au sol. Amir souffle par le nez. Doux. Doux, oui. Tu le vois, le coussin ? Oui, papa. Tu restes ici, Amir ? Oui. Ils restent près de la table. Ça sent l'orange, un peu tiède. Elle est là. Elle est là. Le bois est calme ? Oui, papa. Le ventre d'Amir se desserre. Les épaules descendent un peu. On reste près de la table ? Oui. Tes mains sont au frais ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina a dit stop. Elle a pu s'éloigner. Elle est allée vers maman, l'adulte. Tu as dit stop. Bravo. Tu restes près de moi ? Oui. Le coussin chat est loin. L'horloge fait tic tac.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut jouer, tout de suite. Je joue, maintenant ! Il avance trop vite vers Nina. Le coussin reste collé à sa poitrine. Viens. Nina pousse le coussin. Oh. Le sourire ne revient pas. C'est trop. &lt;emphasis level="moderate"&gt;Stop&lt;/emphasis&gt;. Amir recule d'un pas. Personne ne parle. Il observe le coussin, un instant. Il écoute le bruit de la lampe. Tu veux de l'air, Amir ? Papa reste à la même hauteur. Plus loin. Nina ne dit rien, d'abord. Elle tire le coussin vers elle. Loin. Loin, oui. Merci, Amir. Papa a vu les deux, près du bol. Le coussin colle un peu, sous les doigts. Il est mou. Nina pose le coussin au sol. Amir souffle par le nez. Doux. Doux, oui. Tu le vois, le coussin ? Oui, papa. Tu restes ici, Amir ? Oui. Ils restent près de la table. Ça sent l'orange, un peu tiède. Elle est là. Elle est là. Le bois est calme ? Oui, papa. Le ventre d'Amir se desserre. Les épaules descendent un peu. On reste près de la table ? Oui. Tes mains sont au frais ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;François a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il a pu s'éloigner. Il est allé vers maman, l'adulte.&lt;/slow&gt; [pause]</t>
+          <t>Amir veut jouer, tout de suite. Je joue, maintenant ! Il avance trop vite vers Nina. Le coussin reste collé à sa poitrine. Viens. Nina pousse le coussin. Oh. Le sourire ne revient pas. C'est trop. &lt;emphasis&gt;Stop&lt;/emphasis&gt;. Amir recule d'un pas. Personne ne parle. Il observe le coussin, un instant. Il écoute le bruit de la lampe. Tu veux de l'air, Amir ? Papa reste à la même hauteur. Plus loin. Nina ne dit rien, d'abord. Elle tire le coussin vers elle. Loin. Loin, oui. Merci, Amir. Papa a vu les deux, près du bol. Le coussin colle un peu, sous les doigts. Il est mou. Nina pose le coussin au sol. Amir souffle par le nez. Doux. Doux, oui. Tu le vois, le coussin ? Oui, papa. Tu restes ici, Amir ? Oui. Ils restent près de la table. Ça sent l'orange, un peu tiède. Elle est là. Elle est là. Le bois est calme ? Oui, papa. Le ventre d'Amir se desserre. Les épaules descendent un peu. On reste près de la table ? Oui. Tes mains sont au frais ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1644,18 +1674,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1678,30 +1708,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>Stop</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1710,10 +1740,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1722,24 +1752,60 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=il_dit_stop_il_recule_d_un_pas; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina a dit stop.
-narrateur|Elle a pu s'éloigner.
-narrateur|Elle est allée vers maman, l'adulte.
-maman|Tu as dit stop.
-maman|Bravo.
-maman|Tu restes près de moi ?
-enfant-f|Oui.
-narrateur|Le coussin chat est loin.
-narrateur|L'horloge fait tic tac.</t>
+          <t>narrateur|Amir veut jouer, tout de suite.
+enfant-m|Je joue, maintenant !
+narrateur|Il avance trop vite vers Nina.
+narrateur|Le coussin reste collé à sa poitrine.
+copine|Viens.
+narrateur|Nina pousse le coussin.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+enfant-m|C'est trop.
+enfant-m|Stop.
+narrateur|Amir recule d'un pas.
+narrateur|Personne ne parle.
+narrateur|Il observe le coussin, un instant.
+narrateur|Il écoute le bruit de la lampe.
+papa|Tu veux de l'air, Amir ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Plus loin.
+narrateur|Nina ne dit rien, d'abord.
+narrateur|Elle tire le coussin vers elle.
+copine|Loin.
+enfant-m|Loin, oui.
+papa|Merci, Amir.
+narrateur|Papa a vu les deux, près du bol.
+maman|Le coussin colle un peu, sous les doigts.
+enfant-m|Il est mou.
+narrateur|Nina pose le coussin au sol.
+narrateur|Amir souffle par le nez.
+copine|Doux.
+enfant-m|Doux, oui.
+papa|Tu le vois, le coussin ?
+enfant-m|Oui, papa.
+maman|Tu restes ici, Amir ?
+enfant-m|Oui.
+narrateur|Ils restent près de la table.
+narrateur|Ça sent l'orange, un peu tiède.
+enfant-m|Elle est là.
+copine|Elle est là.
+papa|Le bois est calme ?
+enfant-m|Oui, papa.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules descendent un peu.
+papa|On reste près de la table ?
+enfant-m|Oui.
+maman|Tes mains sont au frais ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1832,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina s'assoit près de maman. Le canapé est doux. Ton ventre s'est serré. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. Le pain grillé sent encore. Nina souffle une dernière fois. Le coussin chat a des moustaches brodées. Nina le regarde de loin. Il reste là-bas. Toi, tu es ici.</t>
+          <t>Maman pose le petit bol. Le bol est un peu flou. Je joue, maintenant ! Nina lève le coussin. Hop. Le coussin glisse trop près. Il glisse, maintenant ! Amir avance le ventre, trop vite. Puis il s'arrête net. Amir refuse de rester collé. Stop. Amir recule d'un pas. Personne ne dit la suite. Il observe la table, un instant. Il écoute le bruit de la lampe. Sur le mur, un éclat de cadre luit. Là, sur le verre. Plus loin, Nina ? Nina ne dit rien. Elle souffle, puis tire. Il glisse. On pose le coussin ? Oui, papa. Amir pousse le coussin. Nina le pose, sans se presser. Il tient. Il tient. Le jus est froid, Nina ? Un peu. Tu bois, Amir ? Oui, maman. Ils boivent près de la table. Le bois chatouille les poignets. C'est plus facile. La lampe est calme ? Oui, papa. Un rayon passe sur le mur. Il allume le cadre. Nina souffle sur le bol. Le jus. Le jus, oui. Le bol laisse un rond. Un rond d'eau.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina s'assoit près de maman. Le canapé est doux. Ton ventre s'est serré. Tu as écouté. Tu es plus calme, maintenant ? Oui, maman. Le pain grillé sent encore. Nina souffle une dernière fois. Le coussin chat a des moustaches brodées. Nina le regarde de loin. Il reste là-bas. Toi, tu es ici.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pose le petit bol. Le bol est un peu flou. Je joue, maintenant ! Nina lève le coussin. Hop. Le coussin glisse trop près. Il glisse, maintenant ! Amir avance le ventre, trop vite. Puis il s'arrête net. Amir refuse de rester collé. Stop. Amir recule d'un pas. Personne ne dit la suite. Il observe la table, un instant. Il écoute le bruit de la lampe. Sur le mur, un &lt;emphasis level="moderate"&gt;éclat de cadre&lt;/emphasis&gt; luit. Là, sur le verre. Plus loin, Nina ? Nina ne dit rien. Elle souffle, puis tire. Il glisse. On pose le coussin ? Oui, papa. Amir pousse le coussin. Nina le pose, sans se presser. Il tient. Il tient. Le jus est froid, Nina ? Un peu. Tu bois, Amir ? Oui, maman. Ils boivent près de la table. Le bois chatouille les poignets. C'est plus facile. La lampe est calme ? Oui, papa. Un rayon passe sur le mur. Il allume le cadre. Nina souffle sur le bol. Le jus. Le jus, oui. Le bol laisse un rond. Un rond d'eau.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;François s'assoit près de maman. Le canapé est doux.&lt;/slow&gt; [pause]</t>
+          <t>Maman pose le petit bol. Le bol est un peu flou. Je joue, maintenant ! Nina lève le coussin. Hop. Le coussin glisse trop près. Il glisse, maintenant ! Amir avance le ventre, trop vite. Puis il s'arrête net. Amir refuse de rester collé. Stop. Amir recule d'un pas. Personne ne dit la suite. Il observe la table, un instant. Il écoute le bruit de la lampe. Sur le mur, un &lt;emphasis&gt;éclat de cadre&lt;/emphasis&gt; luit. Là, sur le verre. Plus loin, Nina ? Nina ne dit rien. Elle souffle, puis tire. Il glisse. On pose le coussin ? Oui, papa. Amir pousse le coussin. Nina le pose, sans se presser. Il tient. Il tient. Le jus est froid, Nina ? Un peu. Tu bois, Amir ? Oui, maman. Ils boivent près de la table. Le bois chatouille les poignets. C'est plus facile. La lampe est calme ? Oui, papa. Un rayon passe sur le mur. Il allume le cadre. Nina souffle sur le bol. Le jus. Le jus, oui. Le bol laisse un rond. Un rond d'eau. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,18 +1889,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1855,28 +1921,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cadre</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1885,10 +1955,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1897,23 +1967,58 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_coussin_glisse_il_dit_stop_encore; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina s'assoit près de maman.
-narrateur|Le canapé est doux.
-maman|Ton ventre s'est serré.
-maman|Tu as écouté.
-maman|Tu es plus calme, maintenant ?
-enfant-f|Oui, maman.
-narrateur|Le pain grillé sent encore.
-narrateur|Nina souffle une dernière fois.
-narrateur|Le coussin chat a des moustaches brodées.
-narrateur|Nina le regarde de loin.
-maman|Il reste là-bas.
-maman|Toi, tu es ici.</t>
+          <t>narrateur|Maman pose le petit bol.
+narrateur|Le bol est un peu flou.
+enfant-m|Je joue, maintenant !
+narrateur|Nina lève le coussin.
+copine|Hop.
+narrateur|Le coussin glisse trop près.
+enfant-m|Il glisse, maintenant !
+narrateur|Amir avance le ventre, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de rester collé.
+enfant-m|Stop.
+narrateur|Amir recule d'un pas.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la table, un instant.
+narrateur|Il écoute le bruit de la lampe.
+narrateur|Sur le mur, un éclat de cadre luit.
+enfant-m|Là, sur le verre.
+enfant-m|Plus loin, Nina ?
+narrateur|Nina ne dit rien.
+narrateur|Elle souffle, puis tire.
+copine|Il glisse.
+papa|On pose le coussin ?
+enfant-m|Oui, papa.
+narrateur|Amir pousse le coussin.
+narrateur|Nina le pose, sans se presser.
+enfant-m|Il tient.
+copine|Il tient.
+papa|Le jus est froid, Nina ?
+copine|Un peu.
+maman|Tu bois, Amir ?
+enfant-m|Oui, maman.
+narrateur|Ils boivent près de la table.
+narrateur|Le bois chatouille les poignets.
+enfant-m|C'est plus facile.
+papa|La lampe est calme ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le mur.
+enfant-m|Il allume le cadre.
+narrateur|Nina souffle sur le bol.
+copine|Le jus.
+enfant-m|Le jus, oui.
+narrateur|Le bol laisse un rond.
+enfant-m|Un rond d'eau.</t>
         </is>
       </c>
     </row>
@@ -1940,17 +2045,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloignée. Je suis allée vers maman. Bravo.</t>
+          <t>Ils restent près de la table. Maman essuie un peu de jus. Le coussin est loin, papa. Tu l'as vu, toi ? Oui, près du sol. On est bien, ici. Amir tapote le bois du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le coussin est resté, Amir. Oui, avec Nina. Le coussin est resté. Ça sent l'orange, un peu tiède. Et le jus, maman. Oui, dans l'air. L'orange reste dans le bol. Un éclat de cadre tient sur le mur.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je me suis éloignée. Je suis allée vers maman. Bravo.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la table. Maman essuie un peu de jus. Le coussin est loin, papa. Tu l'as vu, toi ? Oui, près du sol. On est bien, ici. Amir tapote le bois du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le coussin est resté, Amir. Oui, avec Nina. Le coussin est resté. Ça sent l'orange, un peu tiède. Et le jus, maman. Oui, dans l'air. L'orange reste dans le bol. Un &lt;emphasis level="moderate"&gt;éclat de cadre&lt;/emphasis&gt; tient sur le mur.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la table. Maman essuie un peu de jus. Le coussin est loin, papa. Tu l'as vu, toi ? Oui, près du sol. On est bien, ici. Amir tapote le bois du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le coussin est resté, Amir. Oui, avec Nina. Le coussin est resté. Ça sent l'orange, un peu tiède. Et le jus, maman. Oui, dans l'air. L'orange reste dans le bol. Un &lt;emphasis&gt;éclat de cadre&lt;/emphasis&gt; tient sur le mur.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1997,7 +2102,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2005,7 +2110,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2017,12 +2122,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2031,14 +2136,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cadre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2050,11 +2159,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2063,27 +2172,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_mur; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit stop.
-enfant-f|Je me suis éloignée.
-enfant-f|Je suis allée vers maman.
-maman|Bravo.</t>
+          <t>narrateur|Ils restent près de la table.
+narrateur|Maman essuie un peu de jus.
+enfant-m|Le coussin est loin, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près du sol.
+maman|On est bien, ici.
+narrateur|Amir tapote le bois du doigt.
+enfant-m|Il a une trace d'eau.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le coussin est resté, Amir.
+enfant-m|Oui, avec Nina.
+copine|Le coussin est resté.
+narrateur|Ça sent l'orange, un peu tiède.
+enfant-m|Et le jus, maman.
+maman|Oui, dans l'air.
+narrateur|L'orange reste dans le bol.
+narrateur|Un éclat de cadre tient sur le mur.</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2161,6 +2288,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>